<commit_message>
feat: implement comprehensive monitoring, evaluation, and reporting system including templates and workflow management
</commit_message>
<xml_diff>
--- a/resources/templates/Template Laporan Rencana Tindak Lanjut FST.xlsx
+++ b/resources/templates/Template Laporan Rencana Tindak Lanjut FST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SiGKM\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AAA0489-1E0B-462C-BEDB-1CF38042504D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1E4931-6E85-4639-B727-55098820A2F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C266800C-3CB8-40EA-98D9-08D621FB4B15}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>KEMENTERIAN PENDIDIKAN TINGGI, SAINS, DAN TEKNOLOGI</t>
   </si>
@@ -110,6 +110,12 @@
   </si>
   <si>
     <t xml:space="preserve">                                                                                                                       (CLARISSA ELFIRA AMOS PAH, M.T.I)</t>
+  </si>
+  <si>
+    <t>URAIAN REALISASI TINDAK LANJUT</t>
+  </si>
+  <si>
+    <t>WAKTU PELAKSANAAN</t>
   </si>
 </sst>
 </file>
@@ -359,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -388,63 +394,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -453,6 +402,69 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -859,7 +871,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51C7E03-9B20-46C1-B925-A21BC54F25D4}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.54296875" style="3" customWidth="1"/>
@@ -868,152 +880,180 @@
     <col min="4" max="4" width="70.453125" style="3" customWidth="1"/>
     <col min="5" max="5" width="57.1796875" style="3" customWidth="1"/>
     <col min="6" max="6" width="58.54296875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="54.6328125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="48.1796875" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.90625" style="3"/>
+    <col min="7" max="9" width="54.6328125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="48.1796875" style="3" customWidth="1"/>
+    <col min="11" max="16384" width="8.90625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+    </row>
+    <row r="2" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4"/>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-    </row>
-    <row r="3" spans="1:8" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+    </row>
+    <row r="3" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="4"/>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-    </row>
-    <row r="5" spans="1:8" ht="24.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+    </row>
+    <row r="5" spans="1:10" ht="24.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-    </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+    </row>
+    <row r="6" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
-    </row>
-    <row r="7" spans="1:8" ht="16.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+    </row>
+    <row r="7" spans="1:10" ht="16.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-    </row>
-    <row r="8" spans="1:8" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="12" t="s">
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+    </row>
+    <row r="8" spans="1:10" ht="28.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-    </row>
-    <row r="9" spans="1:8" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="13" t="s">
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+    </row>
+    <row r="9" spans="1:10" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-    </row>
-    <row r="10" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+    </row>
+    <row r="10" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="18"/>
-      <c r="E10" s="23" t="s">
+      <c r="D10" s="27"/>
+      <c r="E10" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-    </row>
-    <row r="11" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="14" t="s">
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="32"/>
+    </row>
+    <row r="11" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="33" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="33" t="s">
+        <v>25</v>
+      </c>
+      <c r="J11" s="19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="25"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="19"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="7">
         <v>1</v>
       </c>
@@ -1035,107 +1075,113 @@
       <c r="G13" s="9">
         <v>12</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E17"/>
-      <c r="F17" s="32" t="s">
+      <c r="F17" s="13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E18"/>
       <c r="F18"/>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E19"/>
       <c r="F19"/>
     </row>
-    <row r="20" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B20" s="29" t="s">
+    <row r="20" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B20" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-    </row>
-    <row r="21" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B21" s="29" t="s">
+      <c r="C20" s="11"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+    </row>
+    <row r="21" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B21" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30" t="s">
+      <c r="C21" s="11"/>
+      <c r="D21" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F21" s="31" t="s">
+      <c r="F21" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B22" s="29"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="F22" s="31"/>
-    </row>
-    <row r="23" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B23" s="29"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="F23" s="31"/>
-    </row>
-    <row r="24" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B24" s="29"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="F24" s="31"/>
-    </row>
-    <row r="25" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B25" s="29"/>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="F25" s="31"/>
-    </row>
-    <row r="26" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B26" s="29"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
-      <c r="F26" s="31"/>
-    </row>
-    <row r="27" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B27" s="29" t="s">
+    <row r="22" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B22" s="10"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="F22" s="12"/>
+    </row>
+    <row r="23" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B23" s="10"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="F23" s="12"/>
+    </row>
+    <row r="24" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B24" s="10"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="F24" s="12"/>
+    </row>
+    <row r="25" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B25" s="10"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="F25" s="12"/>
+    </row>
+    <row r="26" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B26" s="10"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="F26" s="12"/>
+    </row>
+    <row r="27" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B27" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30" t="s">
+      <c r="C27" s="11"/>
+      <c r="D27" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="F27" s="31" t="s">
+      <c r="F27" s="12" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="D2:H2"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B9:H9"/>
+  <mergeCells count="19">
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="D7:J7"/>
+    <mergeCell ref="B8:J8"/>
+    <mergeCell ref="B9:J9"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="C10:D12"/>
-    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="E10:J10"/>
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="D1:J1"/>
+    <mergeCell ref="D2:J2"/>
+    <mergeCell ref="D3:J3"/>
+    <mergeCell ref="D4:J4"/>
+    <mergeCell ref="D5:J5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="122" scale="72" orientation="landscape" r:id="rId1"/>

</xml_diff>